<commit_message>
QA Execution Done Dec-30
</commit_message>
<xml_diff>
--- a/March_Release_SCB/Cypress/fixtures/AgencyTemplate.xlsx
+++ b/March_Release_SCB/Cypress/fixtures/AgencyTemplate.xlsx
@@ -466,10 +466,10 @@
         <v/>
       </c>
       <c r="C2" t="str">
-        <v>626040</v>
+        <v>701863</v>
       </c>
       <c r="D2" t="str">
-        <v>Pearl</v>
+        <v>Janiya</v>
       </c>
       <c r="E2" t="str">
         <v>2256</v>
@@ -499,10 +499,10 @@
         <v>wiki field</v>
       </c>
       <c r="N2" t="str">
-        <v>8748511337</v>
+        <v>1477435206</v>
       </c>
       <c r="O2" t="str">
-        <v>pearl@yopmail.com</v>
+        <v>janiya@yopmail.com</v>
       </c>
       <c r="P2" t="str">
         <v>12-10-2022</v>
@@ -514,7 +514,7 @@
         <v>10-10-2032</v>
       </c>
       <c r="S2" t="str">
-        <v>Bulk upload</v>
+        <v>Bulk upl$%56oad</v>
       </c>
     </row>
   </sheetData>

</xml_diff>